<commit_message>
cho phép đổi quyền, sửa đổi thông tin cá nhân
</commit_message>
<xml_diff>
--- a/client/public/templates/Mau_Import_Nhan_Vien_Z176.xlsx
+++ b/client/public/templates/Mau_Import_Nhan_Vien_Z176.xlsx
@@ -509,7 +509,7 @@
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
@@ -582,7 +582,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Công nghệ thông tin</t>
+          <t>Công nghệ thông tin {Hành chính - Nhân sự}</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -936,6 +936,90 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>5. Phòng ban kiêm nhiệm (một nhân viên làm ở nhiều phòng)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>• Ghi ngay trong cột «Phòng ban» theo dạng:  Tên phòng chính {Phòng kiêm nhiệm 1; Phòng kiêm nhiệm 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ví dụ: Tài chính-kế toán {Kiểm kho; Chính trị} → phòng chính là Tài chính-kế toán, kiêm nhiệm Kiểm kho và Chính trị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>• Phòng chính ghi NGOÀI dấu { }, các phòng kiêm nhiệm ghi TRONG { }, ngăn cách nhau bằng dấu chấm phẩy ";" (không dùng dấu phẩy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>• Không có phòng kiêm nhiệm thì chỉ ghi tên phòng chính. Nếu ghi { } nhưng để trống, dòng vẫn được nhập bình thường (coi như không có</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  kiêm nhiệm) và hệ thống hiện cảnh báo ở bước xem trước để bạn kiểm tra lại.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>• Phòng kiêm nhiệm không được trùng phòng chính, không được ghi trùng nhau, và phải có đủ cặp { } (thiếu dấu } sẽ báo lỗi dòng đó).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>• MỌI phòng ban (cả chính lẫn kiêm nhiệm) đều phải có Mã phòng ban. Phòng nào chưa có mã sẽ được liệt kê ở bước xem trước để bạn nhập mã</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  trước khi xác nhận. Phòng ban mới chỉ được tạo sau khi bấm 'Xác nhận nhập' — gõ sai tên sẽ thấy ngay là 'phòng ban MỚI' ở bước xem trước.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>• Khi cập nhật nhân viên đã có: dòng KHÔNG có { } thì GIỮ NGUYÊN phòng kiêm nhiệm hiện có; dòng có { } liệt kê phòng thì thay bằng danh sách mới.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>• Mỗi kỳ thi, nhân viên chọn 1 vai trò (phòng chính hoặc 1 phòng kiêm nhiệm) trên màn hình thí sinh trước khi vào thi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>• Dòng 2 trong sheet 'NhanVien' là ví dụ: Công nghệ thông tin {Hành chính - Nhân sự}.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>